<commit_message>
Update break-even analysis: 20-year horizon, terminology, WTP wording
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dist/downloads/breakeven_calc.xlsx
+++ b/dist/downloads/breakeven_calc.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DA21998-5543-4F57-941F-2A3B8FEC5132}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E676F176-CC23-42C3-8912-799FC8AE6B68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -151,9 +151,6 @@
     <t>HTN management per patient (e.g. age 50–70)</t>
   </si>
   <si>
-    <t xml:space="preserve">  C.  Model Parameters — Relative_value_to_PI  (pre-filled from factorial analysis)</t>
-  </si>
-  <si>
     <t>Scenario</t>
   </si>
   <si>
@@ -265,9 +262,6 @@
     <t>Custom (from Assumptions)</t>
   </si>
   <si>
-    <t xml:space="preserve">  2.  Required QALY Gain per Patient per Year  (at CADTH C$50,000/QALY threshold)</t>
-  </si>
-  <si>
     <t>Required QALY — low</t>
   </si>
   <si>
@@ -290,13 +284,6 @@
   </si>
   <si>
     <t>RV(TF=High)</t>
-  </si>
-  <si>
-    <t>Relative gain
-(×VOI(PI))</t>
-  </si>
-  <si>
-    <t>VOI(PI) (QALYs)</t>
   </si>
   <si>
     <t>Absolute QALY
@@ -310,9 +297,6 @@
     <t>Tx horizon (yr)</t>
   </si>
   <si>
-    <t xml:space="preserve">  4.  Break-Even Verdict — Required vs. Implied QALY Gain</t>
-  </si>
-  <si>
     <t>Compares the most conservative implied QALY gain (HF=Optimal) to the required threshold for each deployment scenario. "Multiple" = Implied annualized gain / Required mid QALY. Values ≥1 confirm break-even.</t>
   </si>
   <si>
@@ -344,9 +328,6 @@
 (High Δ_H)</t>
   </si>
   <si>
-    <t>Verdict</t>
-  </si>
-  <si>
     <t xml:space="preserve">  5.  Sensitivity — What V(PI) would be needed to just break even?</t>
   </si>
   <si>
@@ -372,6 +353,25 @@
   </si>
   <si>
     <t>V(PI) (entered)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  C.  Model Parameters — Relative_value_to_PI  (pre-filled from factorial analysis)- from Excel file "analysis1_factor_summary" and "df_glm_with_pi"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  4.  Break-Even verification — Required vs. Implied QALY Gain</t>
+  </si>
+  <si>
+    <t>verification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relative gain
+</t>
+  </si>
+  <si>
+    <t>delta(PI) (QALYs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  2.  Required QALY Gain per Patient per Year  (at C$50,000/QALY threshold)</t>
   </si>
 </sst>
 </file>
@@ -386,7 +386,7 @@
     <numFmt numFmtId="168" formatCode="0.000000"/>
     <numFmt numFmtId="169" formatCode="#,##0.0\×"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -496,6 +496,20 @@
       <name val="Arial"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -574,7 +588,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -644,29 +658,38 @@
     <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -944,64 +967,64 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" s="26" t="s">
+      <c r="A4" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="26"/>
-      <c r="C4" s="26"/>
-      <c r="D4" s="26"/>
-      <c r="E4" s="26"/>
+      <c r="B4" s="27"/>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="27"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="33" t="s">
+      <c r="B5" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="33"/>
-      <c r="D5" s="33"/>
-      <c r="E5" s="33"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="29"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="33"/>
-      <c r="D7" s="33"/>
-      <c r="E7" s="33"/>
+      <c r="C7" s="29"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="29"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="6"/>
@@ -1011,13 +1034,13 @@
       <c r="E9" s="6"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" s="26" t="s">
+      <c r="A10" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="26"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
+      <c r="B10" s="27"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
@@ -1029,10 +1052,10 @@
       <c r="C11" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="31" t="s">
+      <c r="D11" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="E11" s="31"/>
+      <c r="E11" s="30"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="8" t="s">
@@ -1044,10 +1067,10 @@
       <c r="C12" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="28" t="s">
+      <c r="D12" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="E12" s="28"/>
+      <c r="E12" s="26"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="8" t="s">
@@ -1059,10 +1082,10 @@
       <c r="C13" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D13" s="28" t="s">
+      <c r="D13" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="E13" s="28"/>
+      <c r="E13" s="26"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="8" t="s">
@@ -1074,10 +1097,10 @@
       <c r="C14" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="D14" s="28" t="s">
+      <c r="D14" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="E14" s="28"/>
+      <c r="E14" s="26"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="8" t="s">
@@ -1089,10 +1112,10 @@
       <c r="C15" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="D15" s="28" t="s">
+      <c r="D15" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="E15" s="28"/>
+      <c r="E15" s="26"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="11" t="s">
@@ -1105,10 +1128,10 @@
       <c r="C16" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D16" s="28" t="s">
+      <c r="D16" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="E16" s="28"/>
+      <c r="E16" s="26"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="11" t="s">
@@ -1121,10 +1144,10 @@
       <c r="C17" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D17" s="28" t="s">
+      <c r="D17" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="E17" s="28"/>
+      <c r="E17" s="26"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="6"/>
@@ -1134,13 +1157,13 @@
       <c r="E19" s="6"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" s="26" t="s">
+      <c r="A20" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="26"/>
-      <c r="C20" s="26"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="26"/>
+      <c r="B20" s="27"/>
+      <c r="C20" s="27"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="7" t="s">
@@ -1152,10 +1175,10 @@
       <c r="C21" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D21" s="31" t="s">
+      <c r="D21" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="E21" s="31"/>
+      <c r="E21" s="30"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="8" t="s">
@@ -1167,10 +1190,10 @@
       <c r="C22" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D22" s="28" t="s">
+      <c r="D22" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="E22" s="28"/>
+      <c r="E22" s="26"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="8" t="s">
@@ -1182,25 +1205,25 @@
       <c r="C23" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="D23" s="28" t="s">
+      <c r="D23" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="E23" s="28"/>
+      <c r="E23" s="26"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="8" t="s">
         <v>37</v>
       </c>
       <c r="B24" s="13">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C24" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D24" s="28" t="s">
+      <c r="D24" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="E24" s="28"/>
+      <c r="E24" s="26"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="6"/>
@@ -1210,26 +1233,26 @@
       <c r="E26" s="6"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A27" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="B27" s="26"/>
-      <c r="C27" s="26"/>
-      <c r="D27" s="26"/>
-      <c r="E27" s="26"/>
+      <c r="A27" s="27" t="s">
+        <v>104</v>
+      </c>
+      <c r="B27" s="27"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="27"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="C28" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="D28" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>43</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>30</v>
@@ -1237,7 +1260,7 @@
     </row>
     <row r="29" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B29" s="14">
         <v>0.93979999999999997</v>
@@ -1250,12 +1273,12 @@
         <v>5.4999999999999938E-2</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B30" s="14">
         <v>0.89590000000000003</v>
@@ -1268,12 +1291,12 @@
         <v>0.14129999999999998</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B31" s="14">
         <v>0.83089999999999997</v>
@@ -1286,12 +1309,12 @@
         <v>0.13090000000000002</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B32" s="14">
         <v>0.88890000000000002</v>
@@ -1304,7 +1327,7 @@
         <v>0.10909999999999997</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
@@ -1315,107 +1338,107 @@
       <c r="E34" s="6"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A35" s="26" t="s">
+      <c r="A35" s="27" t="s">
+        <v>51</v>
+      </c>
+      <c r="B35" s="27"/>
+      <c r="C35" s="27"/>
+      <c r="D35" s="27"/>
+      <c r="E35" s="27"/>
+    </row>
+    <row r="36" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="32" t="s">
         <v>52</v>
       </c>
-      <c r="B35" s="26"/>
-      <c r="C35" s="26"/>
-      <c r="D35" s="26"/>
-      <c r="E35" s="26"/>
-    </row>
-    <row r="36" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="30" t="s">
-        <v>53</v>
-      </c>
-      <c r="B36" s="30"/>
-      <c r="C36" s="30"/>
-      <c r="D36" s="30"/>
-      <c r="E36" s="30"/>
+      <c r="B36" s="32"/>
+      <c r="C36" s="32"/>
+      <c r="D36" s="32"/>
+      <c r="E36" s="32"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B37" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C37" s="30" t="s">
         <v>54</v>
       </c>
-      <c r="C37" s="31" t="s">
-        <v>55</v>
-      </c>
-      <c r="D37" s="31"/>
-      <c r="E37" s="31"/>
+      <c r="D37" s="30"/>
+      <c r="E37" s="30"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B38" s="16">
         <v>12.2</v>
       </c>
-      <c r="C38" s="32" t="s">
-        <v>57</v>
-      </c>
-      <c r="D38" s="32"/>
-      <c r="E38" s="32"/>
+      <c r="C38" s="33" t="s">
+        <v>56</v>
+      </c>
+      <c r="D38" s="33"/>
+      <c r="E38" s="33"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B39" s="16">
         <v>10.7</v>
       </c>
-      <c r="C39" s="32" t="s">
-        <v>59</v>
-      </c>
-      <c r="D39" s="32"/>
-      <c r="E39" s="32"/>
+      <c r="C39" s="33" t="s">
+        <v>58</v>
+      </c>
+      <c r="D39" s="33"/>
+      <c r="E39" s="33"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B40" s="15">
         <f>IF(B39="",B38,B38-B39)</f>
         <v>1.5</v>
       </c>
-      <c r="C40" s="29" t="s">
-        <v>61</v>
-      </c>
-      <c r="D40" s="29"/>
-      <c r="E40" s="29"/>
+      <c r="C40" s="31" t="s">
+        <v>60</v>
+      </c>
+      <c r="D40" s="31"/>
+      <c r="E40" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="A10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="A27:E27"/>
     <mergeCell ref="C40:E40"/>
     <mergeCell ref="A35:E35"/>
     <mergeCell ref="A36:E36"/>
     <mergeCell ref="C37:E37"/>
     <mergeCell ref="C38:E38"/>
     <mergeCell ref="C39:E39"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B6:E6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1436,73 +1459,73 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" s="28" t="s">
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" s="26" t="s">
-        <v>64</v>
-      </c>
-      <c r="B4" s="26"/>
-      <c r="C4" s="26"/>
-      <c r="D4" s="26"/>
-      <c r="E4" s="26"/>
-      <c r="F4" s="26"/>
-      <c r="G4" s="26"/>
-      <c r="H4" s="26"/>
-      <c r="I4" s="26"/>
+      <c r="B4" s="27"/>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+      <c r="I4" s="27"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B6" s="13">
         <v>5</v>
@@ -1533,7 +1556,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B7" s="13">
         <v>5</v>
@@ -1564,7 +1587,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B8" s="13">
         <v>10</v>
@@ -1595,7 +1618,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B9" s="13">
         <v>5</v>
@@ -1626,7 +1649,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B10" s="18">
         <f>Assumptions!B22</f>
@@ -1669,41 +1692,41 @@
       <c r="I12" s="6"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A13" s="26" t="s">
-        <v>77</v>
-      </c>
-      <c r="B13" s="26"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="26"/>
-      <c r="I13" s="26"/>
+      <c r="A13" s="36" t="s">
+        <v>109</v>
+      </c>
+      <c r="B13" s="27"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="27"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="27"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="27"/>
+      <c r="I13" s="27"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="D14" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B15" s="17">
         <f>Results!F6</f>
@@ -1728,7 +1751,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B16" s="17">
         <f>Results!F7</f>
@@ -1753,7 +1776,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B17" s="17">
         <f>Results!F8</f>
@@ -1778,7 +1801,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B18" s="17">
         <f>Results!F9</f>
@@ -1803,7 +1826,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B19" s="17">
         <f>Results!F10</f>
@@ -1838,60 +1861,60 @@
       <c r="I21" s="6"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A22" s="26" t="s">
-        <v>81</v>
-      </c>
-      <c r="B22" s="26"/>
-      <c r="C22" s="26"/>
-      <c r="D22" s="26"/>
-      <c r="E22" s="26"/>
-      <c r="F22" s="26"/>
-      <c r="G22" s="26"/>
-      <c r="H22" s="26"/>
-      <c r="I22" s="26"/>
+      <c r="A22" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="B22" s="27"/>
+      <c r="C22" s="27"/>
+      <c r="D22" s="27"/>
+      <c r="E22" s="27"/>
+      <c r="F22" s="27"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="27"/>
+      <c r="I22" s="27"/>
     </row>
     <row r="23" spans="1:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="25" t="s">
-        <v>82</v>
-      </c>
-      <c r="B23" s="25"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="25"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="25"/>
-      <c r="H23" s="25"/>
-      <c r="I23" s="25"/>
+      <c r="A23" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="B23" s="28"/>
+      <c r="C23" s="28"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="28"/>
+      <c r="F23" s="28"/>
+      <c r="G23" s="28"/>
+      <c r="H23" s="28"/>
+      <c r="I23" s="28"/>
     </row>
     <row r="24" spans="1:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="D24" s="34" t="s">
+        <v>107</v>
+      </c>
+      <c r="E24" s="35" t="s">
+        <v>108</v>
+      </c>
+      <c r="F24" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="G24" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="D24" s="20" t="s">
+      <c r="H24" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F24" s="20" t="s">
-        <v>88</v>
-      </c>
-      <c r="G24" s="20" t="s">
-        <v>89</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B25" s="15">
         <f>Assumptions!B29</f>
@@ -1915,16 +1938,16 @@
       </c>
       <c r="G25" s="22">
         <f>IF(Assumptions!B38="","—",F25/Assumptions!B24)</f>
-        <v>8.24999999999999E-3</v>
+        <v>4.124999999999995E-3</v>
       </c>
       <c r="H25" s="18">
         <f>Assumptions!B24</f>
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B26" s="15">
         <f>Assumptions!B30</f>
@@ -1948,16 +1971,16 @@
       </c>
       <c r="G26" s="22">
         <f>IF(Assumptions!B38="","—",F26/Assumptions!B24)</f>
-        <v>2.1194999999999999E-2</v>
+        <v>1.0597499999999999E-2</v>
       </c>
       <c r="H26" s="18">
         <f>Assumptions!B24</f>
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B27" s="15">
         <f>Assumptions!B31</f>
@@ -1981,16 +2004,16 @@
       </c>
       <c r="G27" s="22">
         <f>IF(Assumptions!B38="","—",F27/Assumptions!B24)</f>
-        <v>1.9635000000000003E-2</v>
+        <v>9.8175000000000016E-3</v>
       </c>
       <c r="H27" s="18">
         <f>Assumptions!B24</f>
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B28" s="15">
         <f>Assumptions!B32</f>
@@ -2014,11 +2037,11 @@
       </c>
       <c r="G28" s="22">
         <f>IF(Assumptions!B38="","—",F28/Assumptions!B24)</f>
-        <v>1.6364999999999998E-2</v>
+        <v>8.1824999999999988E-3</v>
       </c>
       <c r="H28" s="18">
         <f>Assumptions!B24</f>
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
@@ -2033,63 +2056,63 @@
       <c r="I30" s="6"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A31" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="B31" s="26"/>
-      <c r="C31" s="26"/>
-      <c r="D31" s="26"/>
-      <c r="E31" s="26"/>
-      <c r="F31" s="26"/>
-      <c r="G31" s="26"/>
-      <c r="H31" s="26"/>
-      <c r="I31" s="26"/>
+      <c r="A31" s="27" t="s">
+        <v>105</v>
+      </c>
+      <c r="B31" s="27"/>
+      <c r="C31" s="27"/>
+      <c r="D31" s="27"/>
+      <c r="E31" s="27"/>
+      <c r="F31" s="27"/>
+      <c r="G31" s="27"/>
+      <c r="H31" s="27"/>
+      <c r="I31" s="27"/>
     </row>
     <row r="32" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="B32" s="25"/>
-      <c r="C32" s="25"/>
-      <c r="D32" s="25"/>
-      <c r="E32" s="25"/>
-      <c r="F32" s="25"/>
-      <c r="G32" s="25"/>
-      <c r="H32" s="25"/>
-      <c r="I32" s="25"/>
+      <c r="A32" s="28" t="s">
+        <v>87</v>
+      </c>
+      <c r="B32" s="28"/>
+      <c r="C32" s="28"/>
+      <c r="D32" s="28"/>
+      <c r="E32" s="28"/>
+      <c r="F32" s="28"/>
+      <c r="G32" s="28"/>
+      <c r="H32" s="28"/>
+      <c r="I32" s="28"/>
     </row>
     <row r="33" spans="1:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B33" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="C33" s="20" t="s">
+        <v>89</v>
+      </c>
+      <c r="D33" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="E33" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="F33" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="G33" s="20" t="s">
         <v>93</v>
       </c>
-      <c r="C33" s="20" t="s">
+      <c r="H33" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="D33" s="20" t="s">
-        <v>95</v>
-      </c>
-      <c r="E33" s="20" t="s">
-        <v>96</v>
-      </c>
-      <c r="F33" s="20" t="s">
-        <v>97</v>
-      </c>
-      <c r="G33" s="20" t="s">
-        <v>98</v>
-      </c>
-      <c r="H33" s="20" t="s">
-        <v>99</v>
-      </c>
       <c r="I33" s="2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B34" s="19">
         <f>Results!F15</f>
@@ -2097,27 +2120,27 @@
       </c>
       <c r="C34" s="22">
         <f>IF(Assumptions!B38="","—",Results!G25)</f>
-        <v>8.24999999999999E-3</v>
+        <v>4.124999999999995E-3</v>
       </c>
       <c r="D34" s="22">
         <f>IF(Assumptions!B38="","—",Results!G26)</f>
-        <v>2.1194999999999999E-2</v>
+        <v>1.0597499999999999E-2</v>
       </c>
       <c r="E34" s="22">
         <f>IF(Assumptions!B38="","—",Results!G27)</f>
-        <v>1.9635000000000003E-2</v>
+        <v>9.8175000000000016E-3</v>
       </c>
       <c r="F34" s="23">
         <f>IF(OR(Assumptions!B38="",C34="—"),"—",C34/B34)</f>
-        <v>211.53846153846129</v>
+        <v>105.76923076923065</v>
       </c>
       <c r="G34" s="23">
         <f>IF(OR(Assumptions!B38="",C34="—"),"—",D34/B34)</f>
-        <v>543.46153846153845</v>
+        <v>271.73076923076923</v>
       </c>
       <c r="H34" s="23">
         <f>IF(OR(Assumptions!B38="",C34="—"),"—",E34/B34)</f>
-        <v>503.46153846153857</v>
+        <v>251.73076923076928</v>
       </c>
       <c r="I34" s="24" t="str">
         <f>IF(Assumptions!B38="","Enter V(PI)",IF(F34="—","—",IF(F34&gt;=1,"✓ Breaks even","Below threshold")))</f>
@@ -2126,7 +2149,7 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B35" s="19">
         <f>Results!F16</f>
@@ -2134,27 +2157,27 @@
       </c>
       <c r="C35" s="22">
         <f>IF(Assumptions!B38="","—",Results!G25)</f>
-        <v>8.24999999999999E-3</v>
+        <v>4.124999999999995E-3</v>
       </c>
       <c r="D35" s="22">
         <f>IF(Assumptions!B38="","—",Results!G26)</f>
-        <v>2.1194999999999999E-2</v>
+        <v>1.0597499999999999E-2</v>
       </c>
       <c r="E35" s="22">
         <f>IF(Assumptions!B38="","—",Results!G27)</f>
-        <v>1.9635000000000003E-2</v>
+        <v>9.8175000000000016E-3</v>
       </c>
       <c r="F35" s="23">
         <f>IF(OR(Assumptions!B38="",C35="—"),"—",C35/B35)</f>
-        <v>528.84615384615324</v>
+        <v>264.42307692307662</v>
       </c>
       <c r="G35" s="23">
         <f>IF(OR(Assumptions!B38="",C35="—"),"—",D35/B35)</f>
-        <v>1358.6538461538462</v>
+        <v>679.32692307692309</v>
       </c>
       <c r="H35" s="23">
         <f>IF(OR(Assumptions!B38="",C35="—"),"—",E35/B35)</f>
-        <v>1258.6538461538464</v>
+        <v>629.32692307692321</v>
       </c>
       <c r="I35" s="24" t="str">
         <f>IF(Assumptions!B38="","Enter V(PI)",IF(F35="—","—",IF(F35&gt;=1,"✓ Breaks even","Below threshold")))</f>
@@ -2163,7 +2186,7 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B36" s="19">
         <f>Results!F17</f>
@@ -2171,27 +2194,27 @@
       </c>
       <c r="C36" s="22">
         <f>IF(Assumptions!B38="","—",Results!G25)</f>
-        <v>8.24999999999999E-3</v>
+        <v>4.124999999999995E-3</v>
       </c>
       <c r="D36" s="22">
         <f>IF(Assumptions!B38="","—",Results!G26)</f>
-        <v>2.1194999999999999E-2</v>
+        <v>1.0597499999999999E-2</v>
       </c>
       <c r="E36" s="22">
         <f>IF(Assumptions!B38="","—",Results!G27)</f>
-        <v>1.9635000000000003E-2</v>
+        <v>9.8175000000000016E-3</v>
       </c>
       <c r="F36" s="23">
         <f>IF(OR(Assumptions!B38="",C36="—"),"—",C36/B36)</f>
-        <v>1057.6923076923065</v>
+        <v>528.84615384615324</v>
       </c>
       <c r="G36" s="23">
         <f>IF(OR(Assumptions!B38="",C36="—"),"—",D36/B36)</f>
-        <v>2717.3076923076924</v>
+        <v>1358.6538461538462</v>
       </c>
       <c r="H36" s="23">
         <f>IF(OR(Assumptions!B38="",C36="—"),"—",E36/B36)</f>
-        <v>2517.3076923076928</v>
+        <v>1258.6538461538464</v>
       </c>
       <c r="I36" s="24" t="str">
         <f>IF(Assumptions!B38="","Enter V(PI)",IF(F36="—","—",IF(F36&gt;=1,"✓ Breaks even","Below threshold")))</f>
@@ -2200,7 +2223,7 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B37" s="19">
         <f>Results!F18</f>
@@ -2208,27 +2231,27 @@
       </c>
       <c r="C37" s="22">
         <f>IF(Assumptions!B38="","—",Results!G25)</f>
-        <v>8.24999999999999E-3</v>
+        <v>4.124999999999995E-3</v>
       </c>
       <c r="D37" s="22">
         <f>IF(Assumptions!B38="","—",Results!G26)</f>
-        <v>2.1194999999999999E-2</v>
+        <v>1.0597499999999999E-2</v>
       </c>
       <c r="E37" s="22">
         <f>IF(Assumptions!B38="","—",Results!G27)</f>
-        <v>1.9635000000000003E-2</v>
+        <v>9.8175000000000016E-3</v>
       </c>
       <c r="F37" s="23">
         <f>IF(OR(Assumptions!B38="",C37="—"),"—",C37/B37)</f>
-        <v>1057.6923076923065</v>
+        <v>528.84615384615324</v>
       </c>
       <c r="G37" s="23">
         <f>IF(OR(Assumptions!B38="",C37="—"),"—",D37/B37)</f>
-        <v>2717.3076923076924</v>
+        <v>1358.6538461538462</v>
       </c>
       <c r="H37" s="23">
         <f>IF(OR(Assumptions!B38="",C37="—"),"—",E37/B37)</f>
-        <v>2517.3076923076928</v>
+        <v>1258.6538461538464</v>
       </c>
       <c r="I37" s="24" t="str">
         <f>IF(Assumptions!B38="","Enter V(PI)",IF(F37="—","—",IF(F37&gt;=1,"✓ Breaks even","Below threshold")))</f>
@@ -2237,7 +2260,7 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B38" s="19">
         <f>Results!F19</f>
@@ -2245,27 +2268,27 @@
       </c>
       <c r="C38" s="22">
         <f>IF(Assumptions!B38="","—",Results!G25)</f>
-        <v>8.24999999999999E-3</v>
+        <v>4.124999999999995E-3</v>
       </c>
       <c r="D38" s="22">
         <f>IF(Assumptions!B38="","—",Results!G26)</f>
-        <v>2.1194999999999999E-2</v>
+        <v>1.0597499999999999E-2</v>
       </c>
       <c r="E38" s="22">
         <f>IF(Assumptions!B38="","—",Results!G27)</f>
-        <v>1.9635000000000003E-2</v>
+        <v>9.8175000000000016E-3</v>
       </c>
       <c r="F38" s="23">
         <f>IF(OR(Assumptions!B38="",C38="—"),"—",C38/B38)</f>
-        <v>528.84615384615324</v>
+        <v>264.42307692307662</v>
       </c>
       <c r="G38" s="23">
         <f>IF(OR(Assumptions!B38="",C38="—"),"—",D38/B38)</f>
-        <v>1358.6538461538462</v>
+        <v>679.32692307692309</v>
       </c>
       <c r="H38" s="23">
         <f>IF(OR(Assumptions!B38="",C38="—"),"—",E38/B38)</f>
-        <v>1258.6538461538464</v>
+        <v>629.32692307692321</v>
       </c>
       <c r="I38" s="24" t="str">
         <f>IF(Assumptions!B38="","Enter V(PI)",IF(F38="—","—",IF(F38&gt;=1,"✓ Breaks even","Below threshold")))</f>
@@ -2284,72 +2307,72 @@
       <c r="I40" s="6"/>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A41" s="26" t="s">
-        <v>101</v>
-      </c>
-      <c r="B41" s="26"/>
-      <c r="C41" s="26"/>
-      <c r="D41" s="26"/>
-      <c r="E41" s="26"/>
-      <c r="F41" s="26"/>
-      <c r="G41" s="26"/>
-      <c r="H41" s="26"/>
-      <c r="I41" s="26"/>
+      <c r="A41" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="B41" s="27"/>
+      <c r="C41" s="27"/>
+      <c r="D41" s="27"/>
+      <c r="E41" s="27"/>
+      <c r="F41" s="27"/>
+      <c r="G41" s="27"/>
+      <c r="H41" s="27"/>
+      <c r="I41" s="27"/>
     </row>
     <row r="42" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="25" t="s">
-        <v>108</v>
-      </c>
-      <c r="B42" s="25"/>
-      <c r="C42" s="25"/>
-      <c r="D42" s="25"/>
-      <c r="E42" s="25"/>
-      <c r="F42" s="25"/>
-      <c r="G42" s="25"/>
-      <c r="H42" s="25"/>
-      <c r="I42" s="25"/>
+      <c r="A42" s="28" t="s">
+        <v>102</v>
+      </c>
+      <c r="B42" s="28"/>
+      <c r="C42" s="28"/>
+      <c r="D42" s="28"/>
+      <c r="E42" s="28"/>
+      <c r="F42" s="28"/>
+      <c r="G42" s="28"/>
+      <c r="H42" s="28"/>
+      <c r="I42" s="28"/>
     </row>
     <row r="43" spans="1:9" ht="23" x14ac:dyDescent="0.35">
       <c r="A43" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C43" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E43" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="D43" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>109</v>
-      </c>
       <c r="F43" s="2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B44" s="15">
         <f>Results!F15*Assumptions!B24/Results!D25</f>
-        <v>7.0909090909090991E-3</v>
+        <v>1.4181818181818198E-2</v>
       </c>
       <c r="C44" s="15">
         <f>Results!F15*Assumptions!B24/Results!D26</f>
-        <v>2.7600849256900215E-3</v>
+        <v>5.520169851380043E-3</v>
       </c>
       <c r="D44" s="15">
         <f>Results!F15*Assumptions!B24/Results!D27</f>
-        <v>2.9793735676088614E-3</v>
+        <v>5.9587471352177228E-3</v>
       </c>
       <c r="E44" s="15">
         <f>IF(Assumptions!B38="","—",Assumptions!B38)</f>
@@ -2357,32 +2380,32 @@
       </c>
       <c r="F44" s="21">
         <f>IF(Assumptions!B38="","—",E44-B44)</f>
-        <v>12.19290909090909</v>
+        <v>12.185818181818181</v>
       </c>
       <c r="G44" s="21">
         <f>IF(Assumptions!B38="","—",E44-C44)</f>
-        <v>12.197239915074309</v>
+        <v>12.194479830148619</v>
       </c>
       <c r="H44" s="21">
         <f>IF(Assumptions!B38="","—",E44-D44)</f>
-        <v>12.197020626432391</v>
+        <v>12.194041252864782</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B45" s="15">
         <f>Results!F16*Assumptions!B24/Results!D25</f>
-        <v>2.8363636363636395E-3</v>
+        <v>5.6727272727272789E-3</v>
       </c>
       <c r="C45" s="15">
         <f>Results!F16*Assumptions!B24/Results!D26</f>
-        <v>1.1040339702760086E-3</v>
+        <v>2.2080679405520171E-3</v>
       </c>
       <c r="D45" s="15">
         <f>Results!F16*Assumptions!B24/Results!D27</f>
-        <v>1.1917494270435446E-3</v>
+        <v>2.3834988540870892E-3</v>
       </c>
       <c r="E45" s="15">
         <f>IF(Assumptions!B38="","—",Assumptions!B38)</f>
@@ -2390,32 +2413,32 @@
       </c>
       <c r="F45" s="21">
         <f>IF(Assumptions!B38="","—",E45-B45)</f>
-        <v>12.197163636363635</v>
+        <v>12.194327272727271</v>
       </c>
       <c r="G45" s="21">
         <f>IF(Assumptions!B38="","—",E45-C45)</f>
-        <v>12.198895966029724</v>
+        <v>12.197791932059447</v>
       </c>
       <c r="H45" s="21">
         <f>IF(Assumptions!B38="","—",E45-D45)</f>
-        <v>12.198808250572956</v>
+        <v>12.197616501145912</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A46" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B46" s="15">
         <f>Results!F17*Assumptions!B24/Results!D25</f>
-        <v>1.4181818181818197E-3</v>
+        <v>2.8363636363636395E-3</v>
       </c>
       <c r="C46" s="15">
         <f>Results!F17*Assumptions!B24/Results!D26</f>
-        <v>5.5201698513800428E-4</v>
+        <v>1.1040339702760086E-3</v>
       </c>
       <c r="D46" s="15">
         <f>Results!F17*Assumptions!B24/Results!D27</f>
-        <v>5.958747135217723E-4</v>
+        <v>1.1917494270435446E-3</v>
       </c>
       <c r="E46" s="15">
         <f>IF(Assumptions!B38="","—",Assumptions!B38)</f>
@@ -2423,32 +2446,32 @@
       </c>
       <c r="F46" s="21">
         <f>IF(Assumptions!B38="","—",E46-B46)</f>
-        <v>12.198581818181818</v>
+        <v>12.197163636363635</v>
       </c>
       <c r="G46" s="21">
         <f>IF(Assumptions!B38="","—",E46-C46)</f>
-        <v>12.199447983014862</v>
+        <v>12.198895966029724</v>
       </c>
       <c r="H46" s="21">
         <f>IF(Assumptions!B38="","—",E46-D46)</f>
-        <v>12.199404125286478</v>
+        <v>12.198808250572956</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A47" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B47" s="15">
         <f>Results!F18*Assumptions!B24/Results!D25</f>
-        <v>1.4181818181818197E-3</v>
+        <v>2.8363636363636395E-3</v>
       </c>
       <c r="C47" s="15">
         <f>Results!F18*Assumptions!B24/Results!D26</f>
-        <v>5.5201698513800428E-4</v>
+        <v>1.1040339702760086E-3</v>
       </c>
       <c r="D47" s="15">
         <f>Results!F18*Assumptions!B24/Results!D27</f>
-        <v>5.958747135217723E-4</v>
+        <v>1.1917494270435446E-3</v>
       </c>
       <c r="E47" s="15">
         <f>IF(Assumptions!B38="","—",Assumptions!B38)</f>
@@ -2456,32 +2479,32 @@
       </c>
       <c r="F47" s="21">
         <f>IF(Assumptions!B38="","—",E47-B47)</f>
-        <v>12.198581818181818</v>
+        <v>12.197163636363635</v>
       </c>
       <c r="G47" s="21">
         <f>IF(Assumptions!B38="","—",E47-C47)</f>
-        <v>12.199447983014862</v>
+        <v>12.198895966029724</v>
       </c>
       <c r="H47" s="21">
         <f>IF(Assumptions!B38="","—",E47-D47)</f>
-        <v>12.199404125286478</v>
+        <v>12.198808250572956</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B48" s="15">
         <f>Results!F19*Assumptions!B24/Results!D25</f>
-        <v>2.8363636363636395E-3</v>
+        <v>5.6727272727272789E-3</v>
       </c>
       <c r="C48" s="15">
         <f>Results!F19*Assumptions!B24/Results!D26</f>
-        <v>1.1040339702760086E-3</v>
+        <v>2.2080679405520171E-3</v>
       </c>
       <c r="D48" s="15">
         <f>Results!F19*Assumptions!B24/Results!D27</f>
-        <v>1.1917494270435446E-3</v>
+        <v>2.3834988540870892E-3</v>
       </c>
       <c r="E48" s="15">
         <f>IF(Assumptions!B38="","—",Assumptions!B38)</f>
@@ -2489,29 +2512,29 @@
       </c>
       <c r="F48" s="21">
         <f>IF(Assumptions!B38="","—",E48-B48)</f>
-        <v>12.197163636363635</v>
+        <v>12.194327272727271</v>
       </c>
       <c r="G48" s="21">
         <f>IF(Assumptions!B38="","—",E48-C48)</f>
-        <v>12.198895966029724</v>
+        <v>12.197791932059447</v>
       </c>
       <c r="H48" s="21">
         <f>IF(Assumptions!B38="","—",E48-D48)</f>
-        <v>12.198808250572956</v>
+        <v>12.197616501145912</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A23:I23"/>
+    <mergeCell ref="A31:I31"/>
+    <mergeCell ref="A32:I32"/>
+    <mergeCell ref="A41:I41"/>
+    <mergeCell ref="A42:I42"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A4:I4"/>
     <mergeCell ref="A13:I13"/>
     <mergeCell ref="A22:I22"/>
-    <mergeCell ref="A23:I23"/>
-    <mergeCell ref="A31:I31"/>
-    <mergeCell ref="A32:I32"/>
-    <mergeCell ref="A41:I41"/>
-    <mergeCell ref="A42:I42"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>